<commit_message>
Lead-flow proposal (AMS OS, existing website), launch plan, B2B CTAs, register update
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S6zfxMwM7riK18JSe7Qzmo
</commit_message>
<xml_diff>
--- a/marketing/campanhas-registo.xlsx
+++ b/marketing/campanhas-registo.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z199"/>
+  <dimension ref="A1:Z200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -633,7 +633,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>A definir (LinkedIn DM / formulário / e-mail)</t>
+          <t>Formulário B2B (/malerarbeiten-gewerbe/) → AMS OS (brand ams-swiss)</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -651,9 +651,6 @@
           <t>LinkedIn + Instagram</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
           <t>utm_source=linkedin&amp;utm_medium=social&amp;utm_campaign=b2b-2026-01-dirigent</t>
@@ -664,12 +661,6 @@
           <t>Aprovado – aguarda marca</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
       <c r="X2">
         <f>IF(AND(ISNUMBER(O2),ISNUMBER(T2),T2&gt;0),O2/T2,"")</f>
         <v/>
@@ -678,7 +669,6 @@
         <f>IF(AND(ISNUMBER(V2),ISNUMBER(T2),T2&gt;0),V2/T2,"")</f>
         <v/>
       </c>
-      <c r="Z2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -723,7 +713,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>A definir (WhatsApp / formulário / telefone)</t>
+          <t>WhatsApp (código de campanha) ou formulário → AMS OS (brand maler)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -741,9 +731,6 @@
           <t>Instagram + Facebook (+ TikTok)</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
           <t>utm_source=instagram&amp;utm_medium=reel&amp;utm_campaign=b2c-2026-01-untermieter</t>
@@ -751,15 +738,9 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Storyboard para aprovação</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
+          <t>Aguarda autorização de créditos</t>
+        </is>
+      </c>
       <c r="X3">
         <f>IF(AND(ISNUMBER(O3),ISNUMBER(T3),T3&gt;0),O3/T3,"")</f>
         <v/>
@@ -768,7 +749,6 @@
         <f>IF(AND(ISNUMBER(V3),ISNUMBER(T3),T3&gt;0),V3/T3,"")</f>
         <v/>
       </c>
-      <c r="Z3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -813,27 +793,24 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
+          <t>WhatsApp ou formulário → AMS OS (brand maler)</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Pedidos de oferta</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
           <t>A definir</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Pedidos de oferta</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>A definir</t>
-        </is>
-      </c>
       <c r="L4" t="inlineStr">
         <is>
           <t>Instagram + Facebook</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr">
         <is>
           <t>utm_source=meta&amp;utm_medium=paid&amp;utm_campaign=b2c-2026-02-schneemann</t>
@@ -844,12 +821,6 @@
           <t>Pronto</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
       <c r="X4">
         <f>IF(AND(ISNUMBER(O4),ISNUMBER(T4),T4&gt;0),O4/T4,"")</f>
         <v/>
@@ -858,7 +829,6 @@
         <f>IF(AND(ISNUMBER(V4),ISNUMBER(T4),T4&gt;0),V4/T4,"")</f>
         <v/>
       </c>
-      <c r="Z4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -893,7 +863,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>«Wir bringen Ihren Ladenbau in den Takt.» (a rever com regra B)</t>
+          <t>«Wir spielen unseren Part. Auf den Takt genau.»</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -903,27 +873,24 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
+          <t>Formulário B2B → AMS OS</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Reuniões qualificadas</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
           <t>A definir</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Reuniões qualificadas</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>A definir</t>
-        </is>
-      </c>
       <c r="L5" t="inlineStr">
         <is>
           <t>LinkedIn + Instagram</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr">
         <is>
           <t>utm_source=linkedin&amp;utm_medium=video&amp;utm_campaign=b2b-2026-02-sinfonie</t>
@@ -934,12 +901,6 @@
           <t>Demo de som para aprovação</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr"/>
       <c r="X5">
         <f>IF(AND(ISNUMBER(O5),ISNUMBER(T5),T5&gt;0),O5/T5,"")</f>
         <v/>
@@ -948,7 +909,6 @@
         <f>IF(AND(ISNUMBER(V5),ISNUMBER(T5),T5&gt;0),V5/T5,"")</f>
         <v/>
       </c>
-      <c r="Z5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="X6">
@@ -2888,6 +2848,81 @@
       <c r="Y199" s="2">
         <f>IF(AND(ISNUMBER(V199),ISNUMBER(T199),T199&gt;0),V199/T199,"")</f>
         <v/>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>B2B-2026-03</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Der Dirigent – arquitetos/administrações</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Carrossel 5 slides</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>B2B</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>Arquitetos / administrações imobiliárias</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>Aquisição de contratos B2B</t>
+        </is>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>«Ihr Eröffnungstag. Auf den Takt genau.» (adaptar)</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>Projektbesprechung vereinbaren.</t>
+        </is>
+      </c>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>Formulário B2B → AMS OS</t>
+        </is>
+      </c>
+      <c r="J200" t="inlineStr">
+        <is>
+          <t>Reuniões qualificadas</t>
+        </is>
+      </c>
+      <c r="K200" t="inlineStr">
+        <is>
+          <t>A definir</t>
+        </is>
+      </c>
+      <c r="L200" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="M200" t="inlineStr"/>
+      <c r="N200" t="inlineStr"/>
+      <c r="O200" t="inlineStr"/>
+      <c r="P200" t="inlineStr">
+        <is>
+          <t>utm_source=linkedin&amp;utm_medium=social&amp;utm_campaign=b2b-2026-03-dirigent-arch</t>
+        </is>
+      </c>
+      <c r="Q200" t="inlineStr">
+        <is>
+          <t>Ideia</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -2912,7 +2947,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -2960,6 +2995,20 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>CTA B2B: retalho/rollouts «Rollout-Gespräch vereinbaren.»; arquitetos/administrações «Projektbesprechung vereinbaren.»</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Sistema único: AMS OS (Bexio extinto).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
B2C promise is 24 h (website correct): campaigns, rules, register aligned; website correction withdrawn
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S6zfxMwM7riK18JSe7Qzmo
</commit_message>
<xml_diff>
--- a/marketing/campanhas-registo.xlsx
+++ b/marketing/campanhas-registo.xlsx
@@ -708,7 +708,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Jetzt Wintertermin sichern – Offerte innert 48 Stunden</t>
+          <t>Jetzt Wintertermin sichern – Offerte innert 24 Stunden</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -788,7 +788,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Offerte innert 48 Stunden</t>
+          <t>Offerte innert 24 Stunden</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -2911,9 +2911,6 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="M200" t="inlineStr"/>
-      <c r="N200" t="inlineStr"/>
-      <c r="O200" t="inlineStr"/>
       <c r="P200" t="inlineStr">
         <is>
           <t>utm_source=linkedin&amp;utm_medium=social&amp;utm_campaign=b2b-2026-03-dirigent-arch</t>
@@ -2963,7 +2960,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>«Offerte innert 48 Stunden»: apenas B2C residencial. Proibido em B2B.</t>
+          <t>«Offerte innert 24 Stunden»: apenas B2C residencial. Proibido em B2B.</t>
         </is>
       </c>
     </row>

</xml_diff>